<commit_message>
fix: shows err for non-existent tickers; throws err for MockLLM; fix so run.sh rmvs all processes; edit excel;
</commit_message>
<xml_diff>
--- a/Project_Features_and_Roadmap.xlsx
+++ b/Project_Features_and_Roadmap.xlsx
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Skip pipeline if ticker not in SEC</t>
+          <t>Reject non-SEC tickers at front door</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Fail fast: check EDGAR availability before running; return a clear 'no filings' state instead of burning a full LLM run. [user]</t>
+          <t>✅ IMPLEMENTED. Front-door validation: reject symbols that aren't recognized SEC filers BEFORE a job is created. _resolve_snapshot + a GET /api/ticker/&lt;t&gt; endpoint return 404 for unknown tickers (checked vs SEC's cached ticker→CIK map, fail-open if SEC is down); the Landing search validates on submit and shows an inline error. Real filers with no recent 10-K/10-Q still run (fundamental → N/A). [user]</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>N6  Skip if ticker not in SEC</t>
+          <t>N6  Reject non-SEC tickers (front door)</t>
         </is>
       </c>
       <c r="B8" s="17" t="n"/>
@@ -3658,12 +3658,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Running the full multi-agent + debate pipeline on a ticker with no SEC filings wastes minutes of compute + LLM spend for a weak result.</t>
+          <t>✅ IMPLEMENTED. Enqueuing a full multi-agent + debate run for a typo / non-existent symbol wastes minutes of compute + LLM spend. Rejecting at the front door (not mid-pipeline) means no doomed job is ever created.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Before the chain graph, use edgar_ingest to check filing availability; if none, short-circuit with a clear 'unsupported / no filings' status.</t>
+          <t>Validate the ticker against SEC's cached ticker→CIK map: _resolve_snapshot returns 404 before enqueue (the sole enqueue path) + a GET /api/ticker/&lt;t&gt; endpoint the Landing search calls before navigating; fail-open if SEC is unreachable. Valid filers lacking filings still run (empty fundamental).</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>N6 fail-fast, I20 fail-closed, I19 CI→OIDC, N3 Bedrock provider; API auth (I1) started</t>
+          <t>N6 reject non-SEC tickers (done), I20 fail-closed, I19 CI→OIDC, N3 Bedrock provider; API auth (I1) started</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">

</xml_diff>